<commit_message>
Restructure page explication PDF en 3 blocs encadrés + logo
La page était ~80% vide. Ajout de 2 blocs (obligation d'information au
personnel/intérimaires/sous-traitants, rappel dépôt SharePoint + émargement)
en plus du texte existant, dans le même style de zone encadrée qu'ailleurs
dans le document. Logo VMA en grand format et discret, centré en bas de page.
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G308"/>
+  <dimension ref="A1:G313"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11038,6 +11038,191 @@
         </is>
       </c>
     </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>explication_bloc1_titre</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Objet du document</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Purpose of this document</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Doel van dit document</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Ajouté : restructuration page explication en 3 blocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>explication_bloc2_titre</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Obligation d'information</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Duty to inform</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Informatieplicht</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Ajouté : restructuration page explication en 3 blocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>explication_bloc2_texte</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Ce document doit être porté à la connaissance de l'ensemble du personnel vma sud, des intérimaires et des sous-traitants intervenant sur ce chantier, dans le cadre de la procédure d'accueil et d'ouverture de chantier. Cette information est une obligation légale, préalable à toute intervention sur le site.</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>This document must be brought to the attention of all vma sud staff, temporary workers and subcontractors working on this site, as part of the site induction and opening procedure. This information is a legal requirement, to be completed before any work begins on site.</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Dit document moet ter kennis worden gebracht van alle vma sud-personeelsleden, uitzendkrachten en onderaannemers die op deze werf actief zijn, in het kader van de onthaal- en openingsprocedure van de werf. Deze informatieverstrekking is een wettelijke verplichting, voorafgaand aan elke interventie op de werf.</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Ajouté : restructuration page explication en 3 blocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>explication_bloc3_titre</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Dépôt et prise de connaissance</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Filing and acknowledgement</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Indiening en kennisname</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Ajouté : restructuration page explication en 3 blocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>explication_bloc3_texte</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Ce document doit être déposé dans le dossier SharePoint du chantier. La prise de connaissance par chaque intervenant doit être enregistrée par signature sur la page « Émargement » en fin de document.</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>This document must be filed in the site's SharePoint folder. Acknowledgement of having read it must be recorded by each person's signature on the “Attendance sheet” (Émargement) page at the end of the document.</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Dit document moet worden geplaatst in de SharePoint-map van de werf. De kennisname door elke betrokkene moet worden vastgelegd door een handtekening op de pagina 'Aanwezigheidslijst' (Émargement) aan het einde van het document.</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Ajouté : restructuration page explication en 3 blocs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scinder l'adresse du chantier en Rue/N°/Code postal/Ville
Renseignements Généraux : le champ adresse unique devient 4 champs
(rue, numéro, code postal, ville), recomposés en une ligne pour le PDF.

Le code postal ainsi encodé sert désormais d'aide à l'encodage pour la
recherche de l'hôpital le plus proche (Règles spécifiques) : recherche
lancée automatiquement dès qu'il est renseigné, avec un bouton pour la
resynchroniser si l'adresse change ensuite. Le champ reste éditable
indépendamment pour un ajustement manuel.
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G313"/>
+  <dimension ref="A1:G320"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11223,6 +11223,265 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>adresse_rue</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Rue</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Street</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Straat</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Ajouté : scission adresse du chantier en 4 champs</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>adresse_numero</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Ajouté : scission adresse du chantier en 4 champs</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>adresse_code_postal</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Code postal</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Ajouté : scission adresse du chantier en 4 champs</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>adresse_ville</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Ville</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Stad</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Ajouté : scission adresse du chantier en 4 champs</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>hopital_code_postal_utilise</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Infos admin</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Code postal utilisé pour la recherche : {cp} (depuis l'adresse du chantier)</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Postcode used for the search: {cp} (from the site address)</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Postcode gebruikt voor de zoekopdracht: {cp} (van het bouwplaatsadres)</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Ajouté : recherche hôpitaux basée sur l'adresse</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>hopital_code_postal_manquant</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Infos admin</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Renseigne le code postal du chantier dans Renseignements généraux pour lancer la recherche automatique, ou saisis-le ici.</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Fill in the site's postcode in General Information to launch the automatic search, or enter it here.</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Vul de postcode van de bouwplaats in bij Algemene Inlichtingen om de automatische zoekopdracht te starten, of voer deze hier in.</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Ajouté : recherche hôpitaux basée sur l'adresse</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>hopital_reutiliser_code_postal</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Infos admin</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Reprendre le code postal du chantier ({cp})</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Reuse the site's postcode ({cp})</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Postcode van de bouwplaats overnemen ({cp})</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Ajouté : recherche hôpitaux basée sur l'adresse</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scinder Renseignements Généraux en 2 encadrés distincts
"Renseignements" (client, bureau d'architecture, coordinateur sécurité)
et "Adresse chantier" (rue/n°/code postal/ville) deviennent deux cartes
séparées au lieu d'un seul bloc, cohérent avec le principe de zones
encadrées déjà appliqué ailleurs.
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G320"/>
+  <dimension ref="A1:G322"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11482,6 +11482,80 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>renseignements_titre</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Renseignements</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Inlichtingen</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Ajouté : scission Renseignements Généraux en 2 blocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>adresse_chantier_titre</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Rens.gen.</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Adresse chantier</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Adres bouwplaats</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Ajouté : scission Renseignements Généraux en 2 blocs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Permettre au PM d'uploader sa propre image de page de garde
Nouveau champ "Image page de garde" sur l'écran Identification, sous
Numéro/Nom du chantier : upload PNG/JPG (redimensionné/recompressé côté
navigateur avant stockage, pas de backend), avec aperçu et bouton pour
revenir à l'image générique. Prime sur photoCouverture de
entreprise.json à la génération du PDF si renseignée. Stockée en data
URL dans le dossier JSON, donc portée par Enregistrer/Reprendre comme
le reste du dossier.
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G327"/>
+  <dimension ref="A1:G332"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11741,6 +11741,191 @@
         </is>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>identification_image_page_de_garde_titre</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Image page de garde</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Cover page image</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Afbeelding voorblad</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Ajouté : upload d'une image de couverture propre au chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>identification_image_page_de_garde_texte</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Si vous voulez remplacer l'image générique de la page de garde par votre propre image, téléchargez-la ici.</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>If you want to replace the generic cover page image with your own, upload it here.</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Als u de generieke afbeelding op het voorblad wilt vervangen door uw eigen afbeelding, upload deze dan hier.</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Ajouté : upload d'une image de couverture propre au chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>identification_image_page_de_garde_bouton</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Télécharger une image</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Upload an image</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Een afbeelding uploaden</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Ajouté : upload d'une image de couverture propre au chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>identification_image_page_de_garde_reinitialiser</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Revenir à l'image par défaut</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Revert to the default image</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Terug naar de standaardafbeelding</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Ajouté : upload d'une image de couverture propre au chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>identification_image_page_de_garde_erreur</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Fichier invalide : utilisez une image PNG ou JPG.</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Invalid file: please use a PNG or JPG image.</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Ongeldig bestand: gebruik een PNG- of JPG-afbeelding.</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Ajouté : upload d'une image de couverture propre au chantier</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Réduit la largeur des champs Responsable d'approbation + Signature en Annexe 4
Les colonnes Nom/Email/N° GSM du tableau Responsable d'approbation
(ajouté récemment) débordaient horizontalement. Largeurs réduites d'1/3
(15/13/11rem → 10/8.5/7.5rem, min-w 3xl → 32rem).

Annexe 4 : nouveau bloc "Signature" (remplace l'intitulé "Avis" du
document de référence) avec Operations Manager / Project Manager /
Responsable SIPPT, chacun avec un espace pour signer à la main sur le
PDF imprimé.
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G332"/>
+  <dimension ref="A1:G333"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11926,6 +11926,43 @@
         </is>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>annexe4_signature_titre</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Annexe 4</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>manuel</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Handtekening</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Ajouté : bloc signature (Operations Manager/Project Manager/Responsable SIPPT) en Annexe 4, remplace l'ancien intitulé 'Avis' du document de référence</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajoute la case "Tout cocher" par catégorie dans l'analyse de risques abrégée
Coche/décoche d'un coup tous les items non-aggravés de la catégorie (§6
CLAUDE.md). Comportement binaire simple : décocher un item individuellement
fait retomber la case du titre à décochée, pas d'état indéterminé.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFXiTptZrjH4tqXxgg3KiT
</commit_message>
<xml_diff>
--- a/RePSS_UI_Textes_maitre.xlsx
+++ b/RePSS_UI_Textes_maitre.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G333"/>
+  <dimension ref="A1:G334"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11963,6 +11963,38 @@
         </is>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>analyse_tout_cocher</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Analyse de risques</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>n/a (nouveau)</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Tout cocher</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Check all</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Alles aanvinken</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>